<commit_message>
feat(art): jerarquía de tamaños en estaciones — forja 128px, caldero/biblioteca 96px
Adiós al 'mismo cuadro chico': la forja ahora es el horno grande de la
sala (frames 64×64, como la chimenea del mockup), caldero mediano
(48×48) y biblioteca alta (48×48), usando las versiones PixelLab 64 a
resolución completa. Escenas actualizadas coordinadamente (regiones
AtlasTexture + colisiones 52/68/56). Contrato de tamaños documentado en
el Excel (Edificios + Guia_Estilo): la variedad de tamaños es regla.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Maestro.xlsx
+++ b/Catalogo_Maestro.xlsx
@@ -195,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -259,6 +259,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9969,7 +9972,7 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>Cada PNG conserva SIEMPRE sus dimensiones exactas actuales; las escenas usan AtlasTextures con regiones fijas.</t>
+          <t>Los PNG pueden cambiar de tamaño SOLO coordinadamente con su escena (regiones de AtlasTexture + colisión + escala en el mismo commit). Se BUSCA variedad de tamaños entre estaciones (jerarquía visual: forja 128 &gt; caldero/biblioteca 96 &gt; props menores 64) — no todo el mismo cuadro chico.</t>
         </is>
       </c>
     </row>
@@ -20700,9 +20703,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F35" s="21" t="inlineStr">
-        <is>
-          <t>32×32 / 64×64</t>
+      <c r="F35" s="25" t="inlineStr">
+        <is>
+          <t>48×48 (escena ×2 → 96 px)</t>
         </is>
       </c>
       <c r="G35" s="21" t="inlineStr">
@@ -20721,15 +20724,15 @@
           <t>✅ Hecho</t>
         </is>
       </c>
-      <c r="K35" s="21" t="inlineStr">
-        <is>
-          <t>inicial</t>
+      <c r="K35" s="25" t="inlineStr">
+        <is>
+          <t>Jerarquía de tamaños: biblioteca alta (96px pantalla).</t>
         </is>
       </c>
       <c r="L35" s="21" t="inlineStr"/>
       <c r="M35" s="16" t="inlineStr">
         <is>
-          <t>Estantería de madera 32×32 con 3 filas de libros de colores.</t>
+          <t>Estantería alta PixelLab llena de libros de colores (derivada de rs_biblioteca 64).</t>
         </is>
       </c>
     </row>
@@ -20759,9 +20762,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F36" s="21" t="inlineStr">
-        <is>
-          <t>32×32 / 64×64</t>
+      <c r="F36" s="25" t="inlineStr">
+        <is>
+          <t>48×48 ×6 frames (escena ×2 → 96 px)</t>
         </is>
       </c>
       <c r="G36" s="21" t="inlineStr">
@@ -20780,15 +20783,15 @@
           <t>✅ Hecho</t>
         </is>
       </c>
-      <c r="K36" s="21" t="inlineStr">
-        <is>
-          <t>inicial</t>
+      <c r="K36" s="25" t="inlineStr">
+        <is>
+          <t>Jerarquía de tamaños: caldero mediano (96px pantalla).</t>
         </is>
       </c>
       <c r="L36" s="21" t="inlineStr"/>
       <c r="M36" s="16" t="inlineStr">
         <is>
-          <t>Caldero de hierro con brebaje verde burbujeante y llamas debajo (6 frames).</t>
+          <t>Caldero de hierro PixelLab con brebaje dorado burbujeante; 6 frames con burbujas/vapor por código. TAMAÑO MEDIO de la jerarquía.</t>
         </is>
       </c>
     </row>
@@ -20932,9 +20935,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F39" s="21" t="inlineStr">
-        <is>
-          <t>32×32 / 64×64</t>
+      <c r="F39" s="25" t="inlineStr">
+        <is>
+          <t>64×64 ×6 frames (escena ×2 → 128 px)</t>
         </is>
       </c>
       <c r="G39" s="21" t="inlineStr">
@@ -20953,15 +20956,15 @@
           <t>✅ Hecho</t>
         </is>
       </c>
-      <c r="K39" s="21" t="inlineStr">
-        <is>
-          <t>inicial</t>
+      <c r="K39" s="25" t="inlineStr">
+        <is>
+          <t>Jerarquía de tamaños: forja grande (128px pantalla), domina la sala.</t>
         </is>
       </c>
       <c r="L39" s="21" t="inlineStr"/>
       <c r="M39" s="16" t="inlineStr">
         <is>
-          <t>Forja de piedra con boca incandescente que pulsa, chimenea y chispas (6 frames).</t>
+          <t>Gran horno de piedra PixelLab con fuego pulsante, chimenea y yunque; 6 frames con brasas/chispas por código. LA GRANDE de la sala, como la chimenea del mockup.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(art): héroes 128×160 estilo mockup — forja chimenea y gran librería
Estilo oficial registrado: art_reference/mockup_estilo.png es la imagen
norte (Guia_Estilo actualizada). Fórmula validada: pixflux + paleta de
24 colores extraída del mockup (ref/paleta_mockup.png en sd-pixel).
- Forja: chimenea de piedra 64×80 con hogar en arco, yunque, humo
  animado en la chimenea + pulso de brasas (6 frames)
- Biblioteca: librería de pared 64×80 llena de libros y frascos
- Escenas coordinadas (regiones 64×80, colisiones de base)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Maestro.xlsx
+++ b/Catalogo_Maestro.xlsx
@@ -9922,7 +9922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9996,7 +9996,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Púrpuras #3a2058 / #6e3aa0 / #9d6dff / #c89bff — color identidad de la tienda.</t>
+          <t>Púrpuras #3a2058/#6e3aa0/#9d6dff/#c89bff para magia/gemas/UI de campo. INTERIORES según mockup: piedra cálida gris-beige, maderas marrón miel a chocolate, dorados en detalles.</t>
         </is>
       </c>
     </row>
@@ -10124,12 +10124,36 @@
       <c r="B18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Referencia de ESTILO</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>art_reference/mockup_estilo.png — imagen norte del look final (sala de piedra+madera, densidad de props, UI madera/pergamino). TODO asset nuevo se genera con PixelLab bitforge usando un crop de esta imagen como style_image (style_strength ~55-70).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Jerarquía de tamaños</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Variedad deliberada (px pantalla, escena ×2): héroes 128×160+ (forja, biblioteca, alambique central), medianos 96 (caldero, mesas de trabajo), props 48-64, detalles 24-32. Nada de 'todo el mismo cuadro chico'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Generador PIL en ~/Proyectos/sd-pixel/cozy_all/ (un módulo por lote). Regenerar → copiar a godot/art/ → godot --headless --import → validar con movie mode.</t>
         </is>
@@ -20705,7 +20729,7 @@
       </c>
       <c r="F35" s="25" t="inlineStr">
         <is>
-          <t>48×48 (escena ×2 → 96 px)</t>
+          <t>64×80 (escena ×2 → 128×160 px)</t>
         </is>
       </c>
       <c r="G35" s="21" t="inlineStr">
@@ -20726,13 +20750,13 @@
       </c>
       <c r="K35" s="25" t="inlineStr">
         <is>
-          <t>Jerarquía de tamaños: biblioteca alta (96px pantalla).</t>
+          <t>Jerarquía: héroe 128×160. Regenerar con bitforge + style_image del mockup.</t>
         </is>
       </c>
       <c r="L35" s="21" t="inlineStr"/>
       <c r="M35" s="16" t="inlineStr">
         <is>
-          <t>Estantería alta PixelLab llena de libros de colores (derivada de rs_biblioteca 64).</t>
+          <t>Gran librería de pared estilo mockup: alta, llena de libros, frascos y detalles; bitforge con mockup_estilo. Héroe de la sala.</t>
         </is>
       </c>
     </row>
@@ -20937,7 +20961,7 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>64×64 ×6 frames (escena ×2 → 128 px)</t>
+          <t>64×80 ×6 frames (escena ×2 → 128×160 px)</t>
         </is>
       </c>
       <c r="G39" s="21" t="inlineStr">
@@ -20958,13 +20982,13 @@
       </c>
       <c r="K39" s="25" t="inlineStr">
         <is>
-          <t>Jerarquía de tamaños: forja grande (128px pantalla), domina la sala.</t>
+          <t>Jerarquía: héroe 128×160. Regenerar con bitforge + style_image del mockup.</t>
         </is>
       </c>
       <c r="L39" s="21" t="inlineStr"/>
       <c r="M39" s="16" t="inlineStr">
         <is>
-          <t>Gran horno de piedra PixelLab con fuego pulsante, chimenea y yunque; 6 frames con brasas/chispas por código. LA GRANDE de la sala, como la chimenea del mockup.</t>
+          <t>Horno/chimenea de piedra ALTO estilo mockup, fuego pulsante, chimenea hasta arriba; bitforge con mockup_estilo. Héroe de la sala.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(world): Taller como sala PINTADA — el mockup hecho fondo jugable
Técnica definitiva: el propio mockup del usuario repintado por PixelLab
(pixflux init_image strength 250, 3 paneles 320×368) → una ilustración
cohesiva con chimenea, estantes llenos, alambique central brillante,
alfombras, plantas y cristales. Limpieza vía /inpaint: 2 personajes
horneados, 4 letreros con texto gibberish, restos de UI del mockup +
clones locales de suelo. A media resolución con escala ×2 = pitch 2
unificado con personajes y estaciones (adiós sensación de tileset).
Cámara 0.67 (sala completa visible), estaciones sobre la sala pintada.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Maestro.xlsx
+++ b/Catalogo_Maestro.xlsx
@@ -9922,7 +9922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10138,22 +10138,34 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
+          <t>Salas pintadas (diorama)</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Los fondos de sala NO son tilesets: se generan como ilustración con pixflux init_image = crops del mockup (strength 250, 3 paneles 320×368, media resolución + escala ×2 en escena = pitch 2 unificado). Limpieza con /inpaint: personajes horneados, letreros con texto sin sentido, restos de UI. Pipeline en cozy_all/diorama.py + output/pixellab/diorama/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
           <t>Jerarquía de tamaños</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Variedad deliberada (px pantalla, escena ×2): héroes 128×160+ (forja, biblioteca, alambique central), medianos 96 (caldero, mesas de trabajo), props 48-64, detalles 24-32. Nada de 'todo el mismo cuadro chico'.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Generador PIL en ~/Proyectos/sd-pixel/cozy_all/ (un módulo por lote). Regenerar → copiar a godot/art/ → godot --headless --import → validar con movie mode.</t>
         </is>

</xml_diff>

<commit_message>
feat(art): sala Taller VACÍA para decorar + caldero rediseño con animación
Sala vacía: solo paredes de piedra irregulares + suelo de madera pintado
(recortes aleatorios, sin patrón tileset) + puerta arqueada + ventanas
con enredaderas. CERO muebles horneados — el usuario decora con los props
del juego. Compuesta por código (cozy_all/room_empty.py) con piezas
grandes PixelLab. 960×368 escala ×2 = pitch 2.

Caldero rediseñado según referencia del usuario: caldero de hierro
redondo con asas sobre base de troncos, brebaje verde brillante; base
PixelLab (init de la ref) + burbujas y vapor animados por código (6
frames). Reemplaza el caldero morado anterior.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Maestro.xlsx
+++ b/Catalogo_Maestro.xlsx
@@ -10143,7 +10143,7 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>Los fondos de sala NO son tilesets: se generan como ilustración con pixflux init_image = crops del mockup (strength 250, 3 paneles 320×368, media resolución + escala ×2 en escena = pitch 2 unificado). Limpieza con /inpaint: personajes horneados, letreros con texto sin sentido, restos de UI. Pipeline en cozy_all/diorama.py + output/pixellab/diorama/.</t>
+          <t>Los fondos de sala son SOLO estructura VACÍA: paredes de piedra + suelo de madera + puerta + ventanas. NADA de muebles/props horneados — el usuario decora con los props del juego. Compuesto por código (cozy_all/room_empty.py): piezas grandes PixelLab (floor/wall/door/window), pared irregular, suelo por recortes aleatorios (sin patrón tileset), viñeta cálida. 960×368 a escala ×2 = pitch 2 unificado.</t>
         </is>
       </c>
     </row>
@@ -20827,7 +20827,7 @@
       <c r="L36" s="21" t="inlineStr"/>
       <c r="M36" s="16" t="inlineStr">
         <is>
-          <t>Caldero de hierro PixelLab con brebaje dorado burbujeante; 6 frames con burbujas/vapor por código. TAMAÑO MEDIO de la jerarquía.</t>
+          <t>Caldero negro de hierro fundido redondo con asas, sobre base de troncos de madera, brebaje verde brillante burbujeante en la superficie; base PixelLab (ref del usuario), burbujas+vapor animados por código (6 frames). 48×48 → 96px pantalla.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(art): REINICIO de estilo a top-down cartoon Zelda Minish Cap
Cambio de dirección artística: se descarta el enfoque cozy-realista +
salas pintadas. Nuevo norte: tiles 16×16 pequeños tileables (para decorar
con TileMap en el editor), cartoon NO realista, paleta viva extraída de
la referencia. Registrado en Guia_Estilo del Excel + art_reference/
minish_ref.png. Foundation validada: tileset de terreno por código
(grass/dirt/sand/water/path/stone/cliff) seamless con paleta Minish.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Maestro.xlsx
+++ b/Catalogo_Maestro.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +79,11 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00AA2255"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="16">
@@ -195,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -264,6 +269,7 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9922,7 +9928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9938,234 +9944,270 @@
       <c r="B1" s="16" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="B2" s="16" t="inlineStr"/>
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>★ ESTILO ACTUAL (jul 2026)</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>REINICIO a top-down cartoon estilo Zelda: The Minish Cap (art_reference/minish_ref.png). Descarta cozy-realista y salas pintadas.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
+          <t>Tiles Minish</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Tiles 16×16 pequeños, tileables/autotile, para decorar con TileMap en el editor. Generados por CÓDIGO (cozy_all/minish.py) = seamless perfecto. Contorno negro #21181b en objetos; suelos lineless. Cartoon NO realista: colores vivos, shading plano 2-3 tonos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Paleta Minish</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>ref/paleta_minish.png (28 colores): verdes #63ab3e/#8fc84f/#c8d45d, tierra #ab5130/#753027, arena/borde acantilado #feae70/#ffd196, cara acantilado #8e4d57, agua #4fa4b8/#92e8c0, piedra #a3a7c2, flores #f5ffe8/#ffd196/#a02b63. NO usar la paleta arcana vieja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="16" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
           <t>Regla</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Detalle</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Pitch unificado</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>1 píxel de arte = 2 píxeles de pantalla. Assets 64×64 y 40×40 se dibujan a media resolución y se escalan ×2 NEAREST; NPCs 32×48, decoraciones e items se dibujan nativos (sus escenas ya escalan ×2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Dimensiones</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Los PNG pueden cambiar de tamaño SOLO coordinadamente con su escena (regiones de AtlasTexture + colisión + escala en el mismo commit). Se BUSCA variedad de tamaños entre estaciones (jerarquía visual: forja 128 &gt; caldero/biblioteca 96 &gt; props menores 64) — no todo el mismo cuadro chico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Contorno</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Contorno sticker de 1 px color #2b1b35 (violeta cálido, nunca negro puro), dibujado POR DEBAJO de los rellenos.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Paleta arcana</t>
+          <t>Pitch unificado</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Púrpuras #3a2058/#6e3aa0/#9d6dff/#c89bff para magia/gemas/UI de campo. INTERIORES según mockup: piedra cálida gris-beige, maderas marrón miel a chocolate, dorados en detalles.</t>
+          <t>1 píxel de arte = 2 píxeles de pantalla. Assets 64×64 y 40×40 se dibujan a media resolución y se escalan ×2 NEAREST; NPCs 32×48, decoraciones e items se dibujan nativos (sus escenas ya escalan ×2).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Paleta dorada</t>
+          <t>Dimensiones</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Dorados #855a14 / #d27d2c / #f0c060 (+#f8e0a0 highlight) — monedas, magia, madera cálida.</t>
+          <t>Los PNG pueden cambiar de tamaño SOLO coordinadamente con su escena (regiones de AtlasTexture + colisión + escala en el mismo commit). Se BUSCA variedad de tamaños entre estaciones (jerarquía visual: forja 128 &gt; caldero/biblioteca 96 &gt; props menores 64) — no todo el mismo cuadro chico.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Acentos</t>
+          <t>Contorno</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Cyan #6dc2ca, rojo #d04648, azul #597dce, verde #6daa2c + tonos DB16. Piedra #757161/#8595a1, piel #d2aa99, madera #855a14/#a87848.</t>
+          <t>Contorno sticker de 1 px color #2b1b35 (violeta cálido, nunca negro puro), dibujado POR DEBAJO de los rellenos.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Caritas chibi</t>
+          <t>Paleta arcana</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Ojos 2×2 con brillo blanco arriba-izquierda, blush rosa #f0a0b0 a los lados, sonrisita de 2 px. Cabeza grande (~40% de la altura).</t>
+          <t>Púrpuras #3a2058/#6e3aa0/#9d6dff/#c89bff para magia/gemas/UI de campo. INTERIORES según mockup: piedra cálida gris-beige, maderas marrón miel a chocolate, dorados en detalles.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Animación idle</t>
+          <t>Paleta dorada</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>4 frames: bob vertical [0,1,1,0] + parpadeo en frame 3.</t>
+          <t>Dorados #855a14 / #d27d2c / #f0c060 (+#f8e0a0 highlight) — monedas, magia, madera cálida.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Animación walk</t>
+          <t>Acentos</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>6 frames: piernas alternas [-1,-1,0,0,0,0]/[0,0,0,-1,-1,0], bob [0,-1,0,0,-1,0], brazos en swing.</t>
+          <t>Cyan #6dc2ca, rojo #d04648, azul #597dce, verde #6daa2c + tonos DB16. Piedra #757161/#8595a1, piel #d2aa99, madera #855a14/#a87848.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Anim ambiente</t>
+          <t>Caritas chibi</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>Parcelas/caldero/forja: 6 frames horizontales, pulso suave + chispa/burbuja periódica.</t>
+          <t>Ojos 2×2 con brillo blanco arriba-izquierda, blush rosa #f0a0b0 a los lados, sonrisita de 2 px. Cabeza grande (~40% de la altura).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tiles</t>
+          <t>Animación idle</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>Patrones seamless (aritmética modular); verificar repetición 2×2 antes de exportar.</t>
+          <t>4 frames: bob vertical [0,1,1,0] + parpadeo en frame 3.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Animación walk</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>Madera con veta, piedra moteada (hash espacial, no lineal), vidrio translúcido con brillo diagonal 2 px, metal con highlight superior.</t>
+          <t>6 frames: piernas alternas [-1,-1,0,0,0,0]/[0,0,0,-1,-1,0], bob [0,-1,0,0,-1,0], brazos en swing.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Luz</t>
+          <t>Anim ambiente</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>Fuente de luz arriba-izquierda: highlight en esa esquina, sombra propia abajo-derecha.</t>
+          <t>Parcelas/caldero/forja: 6 frames horizontales, pulso suave + chispa/burbuja periódica.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Tiles</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Patrones seamless (aritmética modular); verificar repetición 2×2 antes de exportar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Madera con veta, piedra moteada (hash espacial, no lineal), vidrio translúcido con brillo diagonal 2 px, metal con highlight superior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Fuente de luz arriba-izquierda: highlight en esa esquina, sombra propia abajo-derecha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Transparencias</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Espíritus/vidrio/overlays con alpha 120–230; sombras de contacto alpha ~90.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="16" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="16" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Referencia de ESTILO</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>art_reference/mockup_estilo.png — imagen norte del look final (sala de piedra+madera, densidad de props, UI madera/pergamino). TODO asset nuevo se genera con PixelLab bitforge usando un crop de esta imagen como style_image (style_strength ~55-70).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>Salas pintadas (diorama)</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Los fondos de sala son SOLO estructura VACÍA: paredes de piedra + suelo de madera + puerta + ventanas. NADA de muebles/props horneados — el usuario decora con los props del juego. Compuesto por código (cozy_all/room_empty.py): piezas grandes PixelLab (floor/wall/door/window), pared irregular, suelo por recortes aleatorios (sin patrón tileset), viñeta cálida. 960×368 a escala ×2 = pitch 2 unificado.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Jerarquía de tamaños</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>Variedad deliberada (px pantalla, escena ×2): héroes 128×160+ (forja, biblioteca, alambique central), medianos 96 (caldero, mesas de trabajo), props 48-64, detalles 24-32. Nada de 'todo el mismo cuadro chico'.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>Generador PIL en ~/Proyectos/sd-pixel/cozy_all/ (un módulo por lote). Regenerar → copiar a godot/art/ → godot --headless --import → validar con movie mode.</t>
         </is>

</xml_diff>